<commit_message>
added normalization demo stuff
</commit_message>
<xml_diff>
--- a/Demos/SQL/Normalization/NormalizationDemo.xlsx
+++ b/Demos/SQL/Normalization/NormalizationDemo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JonathanDeLaCruz\Documents\Revature\CGZT-110325\trainer_code\Week3\SQL-Demos\Data Normalization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JonathanDeLaCruz\Documents\Revature\TRNG-2442-NET-Test-Automation\Prep\trainer-code\Demos\SQL\Normalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{409B26CD-3099-4D25-AF68-595D533A9F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD9E8FD-E59A-4420-A1C4-D8822FD79CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD191EF2-E2E2-4C84-ADA3-D38AC6FBC340}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="65">
   <si>
     <t>StudentID</t>
   </si>
@@ -125,9 +125,6 @@
     <t xml:space="preserve">Each record represents one instance of an entity </t>
   </si>
   <si>
-    <t>Student, Course, Instructor?</t>
-  </si>
-  <si>
     <t>Remove repeating groups</t>
   </si>
   <si>
@@ -137,27 +134,6 @@
     <t>Candidate Keys</t>
   </si>
   <si>
-    <t>(StudentID, StudentName, CourseName)</t>
-  </si>
-  <si>
-    <t>(StudentID, CourseID)</t>
-  </si>
-  <si>
-    <t>(StudentID, StudentName, CourseID, CourseName)</t>
-  </si>
-  <si>
-    <t>(Composite Primary Key)</t>
-  </si>
-  <si>
-    <t>We've got The Key - (StudentID, CourseID)</t>
-  </si>
-  <si>
-    <t>StudentID*</t>
-  </si>
-  <si>
-    <t>CourseID*</t>
-  </si>
-  <si>
     <t>First Normal Form</t>
   </si>
   <si>
@@ -173,18 +149,6 @@
     <t>Partial Dependencies:</t>
   </si>
   <si>
-    <t>StudentName depends only on StudentID</t>
-  </si>
-  <si>
-    <t>Instructor Office depends on instructor name</t>
-  </si>
-  <si>
-    <t>CourseName deoends only on CourseID</t>
-  </si>
-  <si>
-    <t>CourseName and Instructor don’t depend on StudentID</t>
-  </si>
-  <si>
     <t>Second Normal Form</t>
   </si>
   <si>
@@ -228,6 +192,45 @@
   </si>
   <si>
     <t>InstructorID (FK)</t>
+  </si>
+  <si>
+    <t>Unnormalized Data</t>
+  </si>
+  <si>
+    <t>MTH202, Calculus I</t>
+  </si>
+  <si>
+    <t>CSE101, Intro to CS</t>
+  </si>
+  <si>
+    <t>PHY105, Classical Mech.</t>
+  </si>
+  <si>
+    <t>Info</t>
+  </si>
+  <si>
+    <t>(StudentName, Instructor)</t>
+  </si>
+  <si>
+    <t>(StudentName, Info)</t>
+  </si>
+  <si>
+    <t>(StudentName, InstructorOffice)</t>
+  </si>
+  <si>
+    <t>StudentName*</t>
+  </si>
+  <si>
+    <t>Instructor*</t>
+  </si>
+  <si>
+    <t>Student name doesn't depend on instructor</t>
+  </si>
+  <si>
+    <t>Grade doesn't depend on instructor</t>
+  </si>
+  <si>
+    <t>Course info doesn’t depend on StudentName</t>
   </si>
 </sst>
 </file>
@@ -259,7 +262,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +272,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -285,11 +300,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -305,6 +326,37 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{44672BDA-7825-4617-A989-8F6D4C15BB7F}" name="Table1" displayName="Table1" ref="C3:H9" totalsRowShown="0">
+  <autoFilter ref="C3:H9" xr:uid="{44672BDA-7825-4617-A989-8F6D4C15BB7F}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{325B0C90-CB10-4CDC-A40A-B3869564DE7F}" name="StudentID"/>
+    <tableColumn id="2" xr3:uid="{D2A2B0B9-94E5-4D71-98D6-1F6230F10B0E}" name="StudentName"/>
+    <tableColumn id="3" xr3:uid="{CB3E0135-C0F5-4D3A-8DAC-FD342F2E3DEE}" name="Info"/>
+    <tableColumn id="4" xr3:uid="{A1A04987-4F9D-4B9C-A4D3-80662F9F64C0}" name="Instructor"/>
+    <tableColumn id="5" xr3:uid="{5428CCEE-7B9F-4232-ADD4-399F3C36A644}" name="InstructorOffice"/>
+    <tableColumn id="6" xr3:uid="{86584CF0-C9E0-4FFF-9F76-6D048FDA6946}" name="Grade"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A91FED13-7FB7-4A3B-BCD2-8FB54BA4FA23}" name="Table2" displayName="Table2" ref="C21:I27" totalsRowShown="0">
+  <autoFilter ref="C21:I27" xr:uid="{A91FED13-7FB7-4A3B-BCD2-8FB54BA4FA23}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{50C94505-F2D1-40A8-862E-1F9411FDBBBE}" name="StudentID"/>
+    <tableColumn id="2" xr3:uid="{B47A1F1D-AC51-4BDE-AE75-5E4CD88459E7}" name="StudentName*"/>
+    <tableColumn id="3" xr3:uid="{35E6A87E-0CFD-4A76-92D0-FC4E9A8ABADF}" name="CourseID"/>
+    <tableColumn id="4" xr3:uid="{03BD6F8C-994A-4C6D-A31C-21F348F5677F}" name="CourseName"/>
+    <tableColumn id="5" xr3:uid="{D1560809-CD3C-49E0-9EAE-B02A6D355F59}" name="Instructor*"/>
+    <tableColumn id="6" xr3:uid="{7CC723C9-FF06-4CAF-AC77-AA7AB7E9F0BB}" name="InstructorOffice"/>
+    <tableColumn id="7" xr3:uid="{9D88B283-81BF-42E1-B222-575892D47DFC}" name="Grade"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -624,19 +676,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D044ED02-15E8-4390-B88F-1DBF12912B02}">
-  <dimension ref="C3:I72"/>
+  <dimension ref="C1:I72"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="17.5546875" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" customWidth="1"/>
+    <col min="5" max="5" width="38.33203125" customWidth="1"/>
     <col min="6" max="6" width="16.44140625" customWidth="1"/>
     <col min="7" max="7" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="21.21875" customWidth="1"/>
     <col min="9" max="9" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="3:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>0</v>
       </c>
@@ -644,22 +708,19 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C4">
         <v>101</v>
       </c>
@@ -667,22 +728,19 @@
         <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C5">
         <v>101</v>
       </c>
@@ -690,22 +748,19 @@
         <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C6">
         <v>102</v>
       </c>
@@ -713,22 +768,19 @@
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C7">
         <v>103</v>
       </c>
@@ -736,22 +788,19 @@
         <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C8">
         <v>103</v>
       </c>
@@ -759,22 +808,19 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="F8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C9">
         <v>103</v>
       </c>
@@ -782,91 +828,78 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>28</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
+      <c r="G14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="G15" t="s">
+    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="H16" s="5"/>
+    </row>
+    <row r="19" spans="3:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="F19" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="H15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="G16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="H17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="3:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="C19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="D21" t="s">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E21" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="F21" t="s">
         <v>3</v>
       </c>
       <c r="G21" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="H21" t="s">
         <v>5</v>
@@ -1015,72 +1048,70 @@
     </row>
     <row r="29" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
-        <v>42</v>
+        <v>34</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="3:9" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="3:9" x14ac:dyDescent="0.3">
       <c r="E33" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="3:9" x14ac:dyDescent="0.3">
       <c r="E34" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="E35" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="3:9" ht="21" x14ac:dyDescent="0.4">
       <c r="E37" s="2" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="G38" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C40" s="3" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C41" s="1" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D41" t="s">
         <v>1</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="G41" t="s">
         <v>3</v>
@@ -1154,15 +1185,15 @@
     </row>
     <row r="46" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C46" s="3" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C47" s="1" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E47" t="s">
         <v>6</v>
@@ -1236,42 +1267,42 @@
     </row>
     <row r="55" spans="3:8" ht="21" x14ac:dyDescent="0.4">
       <c r="E55" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="56" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C56" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C57" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C59" s="3" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C60" s="1" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
         <v>1</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="G60" t="s">
         <v>3</v>
       </c>
       <c r="H60" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
     </row>
     <row r="61" spans="3:8" x14ac:dyDescent="0.3">
@@ -1327,7 +1358,7 @@
     </row>
     <row r="65" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C65" s="3" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>4</v>
@@ -1335,16 +1366,16 @@
     </row>
     <row r="66" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C66" s="1" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E66" t="s">
         <v>6</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="G66" t="s">
         <v>4</v>
@@ -1447,20 +1478,18 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100970BC035301AAD47B5F5A757948CF556" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="776bc5cf192894fc82bd6fc1d893930a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0b98fe4d-4568-4e34-8b21-ba2341edcf62" xmlns:ns4="98c8cb3d-49e7-4737-8eb7-cae46d3ccd57" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b680f66d50dff184f220b222d622a4b2" ns3:_="" ns4:_="">
     <xsd:import namespace="0b98fe4d-4568-4e34-8b21-ba2341edcf62"/>
@@ -1693,6 +1722,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1702,14 +1740,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D9C6CCB-9386-41EB-81BE-EC08B00827FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B95ECDCB-BF4F-436E-989A-661D959E74B6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1724,6 +1754,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D9C6CCB-9386-41EB-81BE-EC08B00827FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>